<commit_message>
Update PostgreSQL requirements and database config
</commit_message>
<xml_diff>
--- a/pingpong_summary_101.xlsx
+++ b/pingpong_summary_101.xlsx
@@ -474,12 +474,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>โอม</t>
+          <t>ภูมิ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>แดง</t>
+          <t>ม่วง</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -492,13 +492,13 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
         <v>2</v>
@@ -510,12 +510,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>อั้ม</t>
+          <t>โอม</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ฟ้า</t>
+          <t>แดง</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -528,13 +528,13 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>

</xml_diff>